<commit_message>
Correçao da questão de reprocessar
</commit_message>
<xml_diff>
--- a/empresas.xlsx
+++ b/empresas.xlsx
@@ -1,31 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Loja\Documents\GitHub\Orcatea-Script\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SAT_RPA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83853BB3-2F52-4A12-96A5-A37A646E8D47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Página1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="128">
   <si>
     <t>Empresa</t>
   </si>
@@ -81,18 +75,352 @@
     <t>Nome</t>
   </si>
   <si>
-    <t>OSNI BOING E CIA LTDA</t>
+    <t>LUCILENE DE AVILA COMERCIO LTDA</t>
+  </si>
+  <si>
+    <t>ROCHA INDUSTRIA E COMERCIO DE ARTEFATOS DE CIMENTO LTDA</t>
+  </si>
+  <si>
+    <t>FARMACIA SÃO RAFAEL LTDA</t>
+  </si>
+  <si>
+    <t>V M B COMERCIO E SERVICOS LTDA</t>
+  </si>
+  <si>
+    <t>AUTO POSTO SHELL LTDA</t>
+  </si>
+  <si>
+    <t>TRANSPORTES E LOGISTICA LTDA</t>
+  </si>
+  <si>
+    <t>J M DISTRIBUIDORES E COMERCIO LTDA</t>
+  </si>
+  <si>
+    <t>COMERCIAL DE ALIMENTOS LTDA</t>
+  </si>
+  <si>
+    <t>ARTE &amp; ESTILO CONFECCOES LTDA</t>
+  </si>
+  <si>
+    <t>R &amp; R SERVICOS DE ESCRITORIO LTDA</t>
+  </si>
+  <si>
+    <t>METALURGICA E USINAGEM LTDA</t>
+  </si>
+  <si>
+    <t>TECH SOLUTION TECNOLOGIA DA INFORMACAO LTDA</t>
+  </si>
+  <si>
+    <t>FARMACIA E DROGARIA CENTRAL LTDA</t>
+  </si>
+  <si>
+    <t>CLINICA MEDICA E ODONTOLOGICA LTDA</t>
+  </si>
+  <si>
+    <t>SUPERMERCADO E MERCEARIA LTDA</t>
+  </si>
+  <si>
+    <t>PADARIA E CONFEITARIA LTDA</t>
+  </si>
+  <si>
+    <t>CONSTRUTORA E EMPREENDIMENTOS LTDA</t>
+  </si>
+  <si>
+    <t>POSTO DE COMBUSTIVEIS LTDA</t>
+  </si>
+  <si>
+    <t>OFICINA MECANICA E AUTO PECAS LTDA</t>
+  </si>
+  <si>
+    <t>GRAFICA E EDITORA LTDA</t>
+  </si>
+  <si>
+    <t>RESTAURANTE E LANCHONETE LTDA</t>
+  </si>
+  <si>
+    <t>LOJAS DE ROUPAS E ACESSORIOS LTDA</t>
+  </si>
+  <si>
+    <t>CONSULTORIA E ASSESSORIA EMPRESARIAL LTDA</t>
+  </si>
+  <si>
+    <t>HOTEL E POUSADA LTDA</t>
+  </si>
+  <si>
+    <t>IMOBILIARIA E CORRETORA LTDA</t>
+  </si>
+  <si>
+    <t>TRANSPORTADORA RAPIDA LTDA</t>
+  </si>
+  <si>
+    <t>AGROPECUARIA E INSUMOS LTDA</t>
+  </si>
+  <si>
+    <t>CORRETORA DE SEGUROS LTDA</t>
+  </si>
+  <si>
+    <t>DISTRIBUIDORA DE BEBIDAS LTDA</t>
+  </si>
+  <si>
+    <t>SALAO DE BELEZA E ESTETICA LTDA</t>
+  </si>
+  <si>
+    <t>PET SHOP E CLINICA VETERINARIA LTDA</t>
+  </si>
+  <si>
+    <t>REDE DE LOJAS DE DEPARTAMENTOS LTDA</t>
+  </si>
+  <si>
+    <t>ACADEMIA E CENTRO ESPORTIVO LTDA</t>
+  </si>
+  <si>
+    <t>ESCOLA E CENTRO DE ENSINO LTDA</t>
+  </si>
+  <si>
+    <t>LABORATORIO DE ANALISES CLINICAS LTDA</t>
+  </si>
+  <si>
+    <t>GRUPO INDUSTRIAL PAULISTA LTDA</t>
+  </si>
+  <si>
+    <t>SOLUCOES EM ENERGIA RENOVAVEL LTDA</t>
+  </si>
+  <si>
+    <t>CASA &amp; CONSTRUCAO MATERIAIS LTDA</t>
+  </si>
+  <si>
+    <t>GUARDSEG SEGURANCA PRIVADA LTDA</t>
+  </si>
+  <si>
+    <t>SERVLIMPA LIMPEZA E PORTARIA LTDA</t>
+  </si>
+  <si>
+    <t>VIAJE MAIS AGENCIA DE VIAGENS LTDA</t>
+  </si>
+  <si>
+    <t>ESTACIONAMENTO E LAVA RAPIDO LTDA</t>
+  </si>
+  <si>
+    <t>INFOCEL COMERCIO DE INFORMATICA LTDA</t>
+  </si>
+  <si>
+    <t>LIVROS &amp; LEITURA EDITORA LTDA</t>
+  </si>
+  <si>
+    <t>BEAUTY DISTRIBUIDORA DE COSMETICOS LTDA</t>
+  </si>
+  <si>
+    <t>AUTOMOTORS COMERCIO DE VEICULOS LTDA</t>
+  </si>
+  <si>
+    <t>ARQENG ENGENHARIA E ARQUITETURA LTDA</t>
+  </si>
+  <si>
+    <t>TEXTIL &amp; MODA INDUSTRIA E COMERCIO LTDA</t>
+  </si>
+  <si>
+    <t>ALIMENTOS &amp; CIA DISTRIBUIDORA LTDA</t>
+  </si>
+  <si>
+    <t>PLASTICOS &amp; EMBALAGENS INDUSTRIA LTDA</t>
+  </si>
+  <si>
+    <t>GRAFICA RAPIDA &amp; COMUNICACAO LTDA</t>
+  </si>
+  <si>
+    <t>SISTEMAS &amp; TECNOLOGIA LTDA</t>
+  </si>
+  <si>
+    <t>CONSULTORIA TRIBUTARIA LTDA</t>
+  </si>
+  <si>
+    <t>CONTABILIDADE &amp; AUDITORIA LTDA</t>
+  </si>
+  <si>
+    <t>LOGISTICA &amp; ARMAZENS GERAIS LTDA</t>
+  </si>
+  <si>
+    <t>IMPORTACAO &amp; EXPORTACAO LTDA</t>
+  </si>
+  <si>
+    <t>43.576.558/0001-22</t>
+  </si>
+  <si>
+    <t>17.881.744/0001-65</t>
+  </si>
+  <si>
+    <t>85.257.319/0001-50</t>
+  </si>
+  <si>
+    <t>12.115.279/0001-38</t>
+  </si>
+  <si>
+    <t>83.414.086/0001-26</t>
+  </si>
+  <si>
+    <t>36.680.479/0001-00</t>
+  </si>
+  <si>
+    <t>12.329.487/0001-30</t>
+  </si>
+  <si>
+    <t>27.665.849/0001-30</t>
+  </si>
+  <si>
+    <t>11.171.338/0001-22</t>
+  </si>
+  <si>
+    <t>11.981.130/0001-79</t>
+  </si>
+  <si>
+    <t>40.414.648/0001-29</t>
+  </si>
+  <si>
+    <t>78.662.020/0001-15</t>
+  </si>
+  <si>
+    <t>08.827.012/0001-04</t>
+  </si>
+  <si>
+    <t>06.024.891/0001-00</t>
+  </si>
+  <si>
+    <t>09.467.868/0001-70</t>
+  </si>
+  <si>
+    <t>06.988.946/0001-94</t>
+  </si>
+  <si>
+    <t>22.583.545/0001-00</t>
+  </si>
+  <si>
+    <t>08.943.124/0001-12</t>
+  </si>
+  <si>
+    <t>76.835.719/0001-04</t>
+  </si>
+  <si>
+    <t>07.018.483/0001-09</t>
+  </si>
+  <si>
+    <t>20.092.970/0001-71</t>
+  </si>
+  <si>
+    <t>32.285.857/0001-91</t>
+  </si>
+  <si>
+    <t>52.124.066/0001-97</t>
+  </si>
+  <si>
+    <t>53.165.803/0001-62</t>
+  </si>
+  <si>
+    <t>41.315.717/0001-00</t>
+  </si>
+  <si>
+    <t>59.561.047/0007-77</t>
+  </si>
+  <si>
+    <t>49.911.169/0001-92</t>
+  </si>
+  <si>
+    <t>82.802.919/0001-63</t>
+  </si>
+  <si>
+    <t>42.602.347/0001-54</t>
+  </si>
+  <si>
+    <t>76.867.30/0001/86</t>
+  </si>
+  <si>
+    <t>76.867.340/0005-00</t>
+  </si>
+  <si>
+    <t>76.867.340/0004-29</t>
+  </si>
+  <si>
+    <t>76.867.340/0003-48</t>
+  </si>
+  <si>
+    <t>76.867.340/0002-67</t>
+  </si>
+  <si>
+    <t>49.129.309/0001-75</t>
+  </si>
+  <si>
+    <t>10.352.560/0001-69</t>
+  </si>
+  <si>
+    <t>09.462.004/0001-66</t>
+  </si>
+  <si>
+    <t>22.133.677/0001-30</t>
+  </si>
+  <si>
+    <t>00.462.179/0001-07</t>
+  </si>
+  <si>
+    <t>46.738.271/0001-40</t>
+  </si>
+  <si>
+    <t>72.452.188/0001-10</t>
+  </si>
+  <si>
+    <t>30.716.386/0001-01</t>
+  </si>
+  <si>
+    <t>66.827.527/0001-00</t>
+  </si>
+  <si>
+    <t>79.848.735/0001-20</t>
+  </si>
+  <si>
+    <t>83.219.097/0001-55</t>
+  </si>
+  <si>
+    <t>83.158.139/0001-95</t>
+  </si>
+  <si>
+    <t>09.512.291/0001-71</t>
+  </si>
+  <si>
+    <t>10.520.923/0001-28</t>
+  </si>
+  <si>
+    <t>19.583.287/0001-58</t>
+  </si>
+  <si>
+    <t>02.708.460/0001-02</t>
+  </si>
+  <si>
+    <t>21.857.514/0001-38</t>
+  </si>
+  <si>
+    <t>22.759.014/0001-26</t>
+  </si>
+  <si>
+    <t>56.072.506/0001-60</t>
+  </si>
+  <si>
+    <t>65.553.070/0001-12</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -110,8 +438,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -124,8 +463,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF9FAFB"/>
+        <bgColor rgb="FFF9FAFB"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -148,30 +493,68 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE0E0E0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE0E0E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE0E0E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE0E0E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFE0E0E0"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -387,11 +770,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="27.140625" customWidth="1"/>
@@ -399,152 +782,774 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
+      <c r="A2" s="7">
+        <v>773</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="7">
+        <v>194</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7">
         <v>349</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
+      <c r="C4" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7">
         <v>350</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B5" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
+      <c r="C5" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7">
         <v>351</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
+      <c r="C6" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7">
         <v>352</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B7" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="2"/>
-    </row>
-    <row r="6" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
+      <c r="C7" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7">
         <v>353</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B8" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="2"/>
-    </row>
-    <row r="7" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
+      <c r="C8" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="7">
         <v>354</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B9" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="2"/>
-    </row>
-    <row r="8" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
+      <c r="C9" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="7">
         <v>355</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B10" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="2"/>
-    </row>
-    <row r="9" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
+      <c r="C10" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="7">
         <v>356</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B11" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="2"/>
-    </row>
-    <row r="10" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
+      <c r="C11" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="7">
         <v>357</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B12" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="2"/>
-    </row>
-    <row r="11" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
+      <c r="C12" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="7">
         <v>358</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B13" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="2"/>
-    </row>
-    <row r="12" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
+      <c r="C13" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="7">
         <v>402</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B14" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="2"/>
-    </row>
-    <row r="13" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
+      <c r="C14" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="7">
         <v>143</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B15" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="2"/>
-    </row>
-    <row r="14" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
+      <c r="C15" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="7">
         <v>165</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B16" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="2"/>
-    </row>
-    <row r="15" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
+      <c r="C16" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="7">
         <v>309</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B17" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="2"/>
-    </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
+      <c r="C17" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="7">
         <v>312</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B18" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="2"/>
+      <c r="C18" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="7">
+        <v>116</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="7">
+        <v>37</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="7">
+        <v>76</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="7">
+        <v>488</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="7">
+        <v>288</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="7">
+        <v>369</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="7">
+        <v>38</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="7">
+        <v>269</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="7">
+        <v>1110</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="7">
+        <v>43</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="7">
+        <v>52</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="7">
+        <v>106</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="7">
+        <v>130</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="7">
+        <v>138</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="7">
+        <v>144</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="7">
+        <v>149</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="7">
+        <v>184</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="7">
+        <v>246</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="7">
+        <v>324</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="7">
+        <v>499</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="7">
+        <v>878</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="7">
+        <v>885</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="7">
+        <v>1105</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="7">
+        <v>1166</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="7">
+        <v>1227</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="7">
+        <v>53</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="7">
+        <v>1120</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="7">
+        <v>300</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="7">
+        <v>834</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="7">
+        <v>828</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="7">
+        <v>786</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="7">
+        <v>474</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="7">
+        <v>862</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="7">
+        <v>459</v>
+      </c>
+      <c r="B52" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="7">
+        <v>153</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="7">
+        <v>221</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="7">
+        <v>137</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="7">
+        <v>813</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="7">
+        <v>189</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="7">
+        <v>406</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="7">
+        <v>1242</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="7">
+        <v>85</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="7">
+        <v>87</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="7">
+        <v>182</v>
+      </c>
+      <c r="B62" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="7">
+        <v>217</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="7">
+        <v>240</v>
+      </c>
+      <c r="B64" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="7">
+        <v>248</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="7">
+        <v>265</v>
+      </c>
+      <c r="B66" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="7">
+        <v>365</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="7">
+        <v>480</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="7">
+        <v>1195</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="7">
+        <v>1220</v>
+      </c>
+      <c r="B70" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>73</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>